<commit_message>
Port OWL class instances as ItemLists; add oa: Motivation/Direction values
owl-to-masp.py: in-namespace instances of a converted class (e.g.
oa:commenting a oa:Motivation) become instance entities listed in one
ItemList per class, and rangeIncludes pointing at that class is replaced
by the ItemList -- the same shape the workflow profile uses for
ComputerLanguage values. Spec, fixture and tests updated.

Regenerated the oa: schema: 13 Motivation and 2 Direction values, used by
motivatedBy, hasPurpose and textDirection. Docs now include the value lists.

masp-validator.js: getEditorValuesForProperty read a non-existent
itemList property, so ItemList members never reached the editor (e.g.
the workflow profile's programmingLanguage list came back empty).

Refs #41

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/schemas/oa/schema-crate/ro-crate-metadata.xlsx
+++ b/schemas/oa/schema-crate/ro-crate-metadata.xlsx
@@ -9,16 +9,19 @@
     <sheet sheetId="3" name="@type=File" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="@type=ResourceDescriptor" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="@type=CreateAction" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="@type=rdfs_Class" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="@type=rdf_Property" state="visible" r:id="rId10"/>
-    <sheet sheetId="8" name="@type=SoftwareApplication" state="visible" r:id="rId11"/>
+    <sheet sheetId="6" name="@type=ItemList" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="@type=rdfs_Class" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="@type=rdf_Property" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="@type=SoftwareApplication" state="visible" r:id="rId12"/>
+    <sheet sheetId="10" name="oa_Direction12" state="visible" r:id="rId13"/>
+    <sheet sheetId="11" name="oa_Motivation13" state="visible" r:id="rId14"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="266">
   <si>
     <t>Name</t>
   </si>
@@ -98,7 +101,7 @@
     <t>"http://www.w3.org/ns/dx/prof/role/schema"</t>
   </si>
   <si>
-    <t>["http://www.w3.org/ns/oa#Annotation", "http://www.w3.org/ns/oa#Choice", "http://www.w3.org/ns/oa#CssSelector", "http://www.w3.org/ns/oa#CssStyle", "http://www.w3.org/ns/oa#DataPositionSelector", "http://www.w3.org/ns/oa#Direction", "http://www.w3.org/ns/oa#FragmentSelector", "http://www.w3.org/ns/oa#HttpRequestState", "http://www.w3.org/ns/oa#Motivation", "http://www.w3.org/ns/oa#RangeSelector", "http://www.w3.org/ns/oa#ResourceSelection", "http://www.w3.org/ns/oa#Selector", "http://www.w3.org/ns/oa#SpecificResource", "http://www.w3.org/ns/oa#State", "http://www.w3.org/ns/oa#Style", "http://www.w3.org/ns/oa#SvgSelector", "http://www.w3.org/ns/oa#TextPositionSelector", "http://www.w3.org/ns/oa#TextQuoteSelector", "http://www.w3.org/ns/oa#TextualBody", "http://www.w3.org/ns/oa#TimeState", "http://www.w3.org/ns/oa#XPathSelector", "http://www.w3.org/ns/oa#annotationService", "http://www.w3.org/ns/oa#bodyValue", "http://www.w3.org/ns/oa#cachedSource", "http://www.w3.org/ns/oa#canonical", "http://www.w3.org/ns/oa#end", "http://www.w3.org/ns/oa#exact", "http://www.w3.org/ns/oa#hasBody", "http://www.w3.org/ns/oa#hasEndSelector", "http://www.w3.org/ns/oa#hasPurpose", "http://www.w3.org/ns/oa#hasScope", "http://www.w3.org/ns/oa#hasSelector", "http://www.w3.org/ns/oa#hasSource", "http://www.w3.org/ns/oa#hasStartSelector", "http://www.w3.org/ns/oa#hasState", "http://www.w3.org/ns/oa#hasTarget", "http://www.w3.org/ns/oa#motivatedBy", "http://www.w3.org/ns/oa#prefix", "http://www.w3.org/ns/oa#processingLanguage", "http://www.w3.org/ns/oa#refinedBy", "http://www.w3.org/ns/oa#renderedVia", "http://www.w3.org/ns/oa#sourceDate", "http://www.w3.org/ns/oa#sourceDateEnd", "http://www.w3.org/ns/oa#sourceDateStart", "http://www.w3.org/ns/oa#start", "http://www.w3.org/ns/oa#styleClass", "http://www.w3.org/ns/oa#styledBy", "http://www.w3.org/ns/oa#suffix", "http://www.w3.org/ns/oa#textDirection", "http://www.w3.org/ns/oa#via"]</t>
+    <t>["#itemlist_Direction", "#itemlist_Motivation", "http://www.w3.org/ns/oa#Annotation", "http://www.w3.org/ns/oa#Choice", "http://www.w3.org/ns/oa#CssSelector", "http://www.w3.org/ns/oa#CssStyle", "http://www.w3.org/ns/oa#DataPositionSelector", "http://www.w3.org/ns/oa#Direction", "http://www.w3.org/ns/oa#FragmentSelector", "http://www.w3.org/ns/oa#HttpRequestState", "http://www.w3.org/ns/oa#Motivation", "http://www.w3.org/ns/oa#RangeSelector", "http://www.w3.org/ns/oa#ResourceSelection", "http://www.w3.org/ns/oa#Selector", "http://www.w3.org/ns/oa#SpecificResource", "http://www.w3.org/ns/oa#State", "http://www.w3.org/ns/oa#Style", "http://www.w3.org/ns/oa#SvgSelector", "http://www.w3.org/ns/oa#TextPositionSelector", "http://www.w3.org/ns/oa#TextQuoteSelector", "http://www.w3.org/ns/oa#TextualBody", "http://www.w3.org/ns/oa#TimeState", "http://www.w3.org/ns/oa#XPathSelector", "http://www.w3.org/ns/oa#annotationService", "http://www.w3.org/ns/oa#bodyValue", "http://www.w3.org/ns/oa#cachedSource", "http://www.w3.org/ns/oa#canonical", "http://www.w3.org/ns/oa#end", "http://www.w3.org/ns/oa#exact", "http://www.w3.org/ns/oa#hasBody", "http://www.w3.org/ns/oa#hasEndSelector", "http://www.w3.org/ns/oa#hasPurpose", "http://www.w3.org/ns/oa#hasScope", "http://www.w3.org/ns/oa#hasSelector", "http://www.w3.org/ns/oa#hasSource", "http://www.w3.org/ns/oa#hasStartSelector", "http://www.w3.org/ns/oa#hasState", "http://www.w3.org/ns/oa#hasTarget", "http://www.w3.org/ns/oa#motivatedBy", "http://www.w3.org/ns/oa#prefix", "http://www.w3.org/ns/oa#processingLanguage", "http://www.w3.org/ns/oa#refinedBy", "http://www.w3.org/ns/oa#renderedVia", "http://www.w3.org/ns/oa#sourceDate", "http://www.w3.org/ns/oa#sourceDateEnd", "http://www.w3.org/ns/oa#sourceDateStart", "http://www.w3.org/ns/oa#start", "http://www.w3.org/ns/oa#styleClass", "http://www.w3.org/ns/oa#styledBy", "http://www.w3.org/ns/oa#suffix", "http://www.w3.org/ns/oa#textDirection", "http://www.w3.org/ns/oa#via"]</t>
   </si>
   <si>
     <t>object</t>
@@ -128,7 +131,31 @@
     <t>"./"</t>
   </si>
   <si>
-    <t>2026-09-28T22:27:58.272020+00:00</t>
+    <t>2026-09-29T01:37:59.575116+00:00</t>
+  </si>
+  <si>
+    <t>itemListElement</t>
+  </si>
+  <si>
+    <t>#itemlist_Direction</t>
+  </si>
+  <si>
+    <t>ItemList</t>
+  </si>
+  <si>
+    <t>Direction values</t>
+  </si>
+  <si>
+    <t>["http://www.w3.org/ns/oa#ltrDirection", "http://www.w3.org/ns/oa#rtlDirection"]</t>
+  </si>
+  <si>
+    <t>#itemlist_Motivation</t>
+  </si>
+  <si>
+    <t>Motivation values</t>
+  </si>
+  <si>
+    <t>["http://www.w3.org/ns/oa#assessing", "http://www.w3.org/ns/oa#bookmarking", "http://www.w3.org/ns/oa#classifying", "http://www.w3.org/ns/oa#commenting", "http://www.w3.org/ns/oa#describing", "http://www.w3.org/ns/oa#editing", "http://www.w3.org/ns/oa#highlighting", "http://www.w3.org/ns/oa#identifying", "http://www.w3.org/ns/oa#linking", "http://www.w3.org/ns/oa#moderating", "http://www.w3.org/ns/oa#questioning", "http://www.w3.org/ns/oa#replying", "http://www.w3.org/ns/oa#tagging"]</t>
   </si>
   <si>
     <t>rdfs:label</t>
@@ -458,7 +485,7 @@
     <t>The purpose served by the resource in the Annotation.</t>
   </si>
   <si>
-    <t>"http://www.w3.org/ns/oa#Motivation"</t>
+    <t>"#itemlist_Motivation"</t>
   </si>
   <si>
     <t>http://www.w3.org/ns/oa#hasScope</t>
@@ -638,7 +665,7 @@
     <t>The direction of the text of the subject resource. There MUST only be one text direction associated with any given resource.</t>
   </si>
   <si>
-    <t>"http://www.w3.org/ns/oa#Direction"</t>
+    <t>"#itemlist_Direction"</t>
   </si>
   <si>
     <t>http://www.w3.org/ns/oa#via</t>
@@ -660,6 +687,141 @@
   </si>
   <si>
     <t>owl-to-masp.py</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/oa#ltrDirection</t>
+  </si>
+  <si>
+    <t>ltrDirection</t>
+  </si>
+  <si>
+    <t>The direction of text that is read from left to right.</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/oa#rtlDirection</t>
+  </si>
+  <si>
+    <t>rtlDirection</t>
+  </si>
+  <si>
+    <t>The direction of text that is read from right to left.</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/oa#assessing</t>
+  </si>
+  <si>
+    <t>assessing</t>
+  </si>
+  <si>
+    <t>The motivation for when the user intends to provide an assessment about the Target resource.</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/oa#bookmarking</t>
+  </si>
+  <si>
+    <t>bookmarking</t>
+  </si>
+  <si>
+    <t>The motivation for when the user intends to create a bookmark to the Target or part thereof.</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/oa#classifying</t>
+  </si>
+  <si>
+    <t>classifying</t>
+  </si>
+  <si>
+    <t>The motivation for when the user intends to that classify the Target as something.</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/oa#commenting</t>
+  </si>
+  <si>
+    <t>commenting</t>
+  </si>
+  <si>
+    <t>The motivation for when the user intends to comment about the Target.</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/oa#describing</t>
+  </si>
+  <si>
+    <t>describing</t>
+  </si>
+  <si>
+    <t>The motivation for when the user intends to describe the Target, as opposed to a comment about them.</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/oa#editing</t>
+  </si>
+  <si>
+    <t>editing</t>
+  </si>
+  <si>
+    <t>The motivation for when the user intends to request a change or edit to the Target resource.</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/oa#highlighting</t>
+  </si>
+  <si>
+    <t>highlighting</t>
+  </si>
+  <si>
+    <t>The motivation for when the user intends to highlight the Target resource or segment of it.</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/oa#identifying</t>
+  </si>
+  <si>
+    <t>identifying</t>
+  </si>
+  <si>
+    <t>The motivation for when the user intends to assign an identity to the Target or identify what is being depicted or described in the Target.</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/oa#linking</t>
+  </si>
+  <si>
+    <t>linking</t>
+  </si>
+  <si>
+    <t>The motivation for when the user intends to link to a resource related to the Target.</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/oa#moderating</t>
+  </si>
+  <si>
+    <t>moderating</t>
+  </si>
+  <si>
+    <t>The motivation for when the user intends to assign some value or quality to the Target.</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/oa#questioning</t>
+  </si>
+  <si>
+    <t>questioning</t>
+  </si>
+  <si>
+    <t>The motivation for when the user intends to ask a question about the Target.</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/oa#replying</t>
+  </si>
+  <si>
+    <t>replying</t>
+  </si>
+  <si>
+    <t>The motivation for when the user intends to reply to a previous statement, either an Annotation or another resource.</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/oa#tagging</t>
+  </si>
+  <si>
+    <t>tagging</t>
+  </si>
+  <si>
+    <t>The motivation for when the user intends to associate a tag with the Target.</t>
   </si>
 </sst>
 </file>
@@ -1113,6 +1275,272 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="4" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D2" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>224</v>
+      </c>
+      <c r="B3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="4" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>230</v>
+      </c>
+      <c r="B3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3" t="s">
+        <v>231</v>
+      </c>
+      <c r="D3" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>233</v>
+      </c>
+      <c r="B4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D4" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>236</v>
+      </c>
+      <c r="B5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" t="s">
+        <v>237</v>
+      </c>
+      <c r="D5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>239</v>
+      </c>
+      <c r="B6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C6" t="s">
+        <v>240</v>
+      </c>
+      <c r="D6" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>242</v>
+      </c>
+      <c r="B7" t="s">
+        <v>77</v>
+      </c>
+      <c r="C7" t="s">
+        <v>243</v>
+      </c>
+      <c r="D7" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>245</v>
+      </c>
+      <c r="B8" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" t="s">
+        <v>246</v>
+      </c>
+      <c r="D8" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>248</v>
+      </c>
+      <c r="B9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D9" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>251</v>
+      </c>
+      <c r="B10" t="s">
+        <v>77</v>
+      </c>
+      <c r="C10" t="s">
+        <v>252</v>
+      </c>
+      <c r="D10" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>254</v>
+      </c>
+      <c r="B11" t="s">
+        <v>77</v>
+      </c>
+      <c r="C11" t="s">
+        <v>255</v>
+      </c>
+      <c r="D11" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>257</v>
+      </c>
+      <c r="B12" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12" t="s">
+        <v>258</v>
+      </c>
+      <c r="D12" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>260</v>
+      </c>
+      <c r="B13" t="s">
+        <v>77</v>
+      </c>
+      <c r="C13" t="s">
+        <v>261</v>
+      </c>
+      <c r="D13" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>263</v>
+      </c>
+      <c r="B14" t="s">
+        <v>77</v>
+      </c>
+      <c r="C14" t="s">
+        <v>264</v>
+      </c>
+      <c r="D14" t="s">
+        <v>265</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B1"/>
@@ -1294,6 +1722,62 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="4" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -1308,415 +1792,415 @@
         <v>4</v>
       </c>
       <c r="C1" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="D1" t="s">
         <v>6</v>
       </c>
       <c r="E1" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="F1" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="B2" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C2" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="D2" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="E2" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C3" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="D3" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="E3" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="F3" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="B4" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D4" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="E4" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="F4" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="B5" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C5" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="D5" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="E5" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="F5" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="B6" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="D6" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="E6" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="F6" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C7" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="D7" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="E7" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C8" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="D8" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="E8" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="F8" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C9" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="D9" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E9" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="F9" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C10" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="D10" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="E10" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="F10" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="B11" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C11" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="D11" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="E11" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F11" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C12" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="D12" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="E12" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="B13" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C13" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="D13" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="E13" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C14" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="D14" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="E14" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="F14" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="B15" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C15" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="D15" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="E15" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="B16" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C16" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="D16" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="E16" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="B17" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C17" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="D17" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="E17" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="F17" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="B18" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C18" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="D18" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="E18" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="F18" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="B19" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C19" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="D19" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="E19" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="F19" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="B20" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C20" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="D20" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="E20" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="B21" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C21" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="D21" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="E21" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="F21" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="B22" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C22" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="D22" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="E22" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="F22" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1725,7 +2209,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1741,620 +2225,620 @@
         <v>4</v>
       </c>
       <c r="C1" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="D1" t="s">
         <v>6</v>
       </c>
       <c r="E1" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="F1" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="G1" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="B2" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C2" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="D2" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="E2" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="B3" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C3" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D3" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="E3" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="F3" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="G3" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B4" t="s">
         <v>121</v>
       </c>
-      <c r="B4" t="s">
-        <v>113</v>
-      </c>
       <c r="C4" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="D4" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="E4" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="F4" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="B5" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C5" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="D5" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="E5" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="B6" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C6" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="D6" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="E6" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="G6" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="B7" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C7" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="D7" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E7" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="G7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="B8" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C8" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="D8" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="E8" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="F8" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="B9" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C9" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="D9" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="E9" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="F9" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="G9" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="B10" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C10" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="D10" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="E10" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="G10" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="B11" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C11" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="D11" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="E11" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="F11" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="B12" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C12" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="D12" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="E12" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="F12" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="G12" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="B13" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C13" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="D13" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="E13" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="F13" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="B14" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C14" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="D14" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="E14" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="F14" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="G14" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="B15" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C15" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="D15" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="E15" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="F15" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="G15" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="B16" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C16" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="D16" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="E16" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="F16" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="B17" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C17" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D17" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="E17" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="F17" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="G17" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="B18" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C18" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="D18" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E18" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="G18" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="B19" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C19" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="D19" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="E19" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="G19" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="B20" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C20" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="D20" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="E20" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="B21" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C21" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="D21" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="E21" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="F21" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="B22" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C22" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="D22" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="E22" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="F22" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="G22" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="B23" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C23" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="D23" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="E23" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="F23" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="G23" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="B24" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C24" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="D24" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="E24" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="F24" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="G24" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="B25" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C25" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="D25" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="E25" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="G25" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="B26" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C26" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="D26" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="E26" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="F26" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="G26" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="B27" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C27" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="D27" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="E27" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="F27" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="G27" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="B28" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C28" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="D28" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="E28" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="G28" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="B29" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C29" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="D29" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="E29" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="G29" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="B30" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C30" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="D30" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="E30" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -2363,7 +2847,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -2382,21 +2866,21 @@
         <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="B2" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="C2" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="D2" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Keep the class alongside the ItemList in ranges; regenerate LexInfo
owl-to-masp.py now adds the ItemList after the class in rangeIncludes
rather than replacing it, so custom instances (e.g. your own
oa:Motivation, which Web Annotation allows) still validate while editors
get the standard values from the list.

Regenerated oa: with this, and regenerated LexInfo with the same command
as 6127002: adds 276 instances in 26 value lists (PartOfSpeech, Case,
Gender, Tense, ...) and extends 25 property ranges. No existing entities
removed. Both schema texts describe the value lists and render them.

Refs #41

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/schemas/oa/schema-crate/ro-crate-metadata.xlsx
+++ b/schemas/oa/schema-crate/ro-crate-metadata.xlsx
@@ -131,7 +131,7 @@
     <t>"./"</t>
   </si>
   <si>
-    <t>2026-09-29T01:37:59.575116+00:00</t>
+    <t>2026-09-29T02:18:30.314542+00:00</t>
   </si>
   <si>
     <t>itemListElement</t>
@@ -485,7 +485,7 @@
     <t>The purpose served by the resource in the Annotation.</t>
   </si>
   <si>
-    <t>"#itemlist_Motivation"</t>
+    <t>["http://www.w3.org/ns/oa#Motivation", "#itemlist_Motivation"]</t>
   </si>
   <si>
     <t>http://www.w3.org/ns/oa#hasScope</t>
@@ -665,7 +665,7 @@
     <t>The direction of the text of the subject resource. There MUST only be one text direction associated with any given resource.</t>
   </si>
   <si>
-    <t>"#itemlist_Direction"</t>
+    <t>["http://www.w3.org/ns/oa#Direction", "#itemlist_Direction"]</t>
   </si>
   <si>
     <t>http://www.w3.org/ns/oa#via</t>

</xml_diff>